<commit_message>
Feat: Tự động tính và điền Tổng tiền bằng chữ sang tiếng Việt vào 3 Sheet
</commit_message>
<xml_diff>
--- a/mau-bang-tien.xlsx
+++ b/mau-bang-tien.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PM-quanlykhoa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB2CB27A-E06C-431D-896D-55FFD86244B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFBD0345-524F-4053-BF84-755CFC278053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{EA3D4609-970D-4ECC-8B52-B6F6CFF039FF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{EA3D4609-970D-4ECC-8B52-B6F6CFF039FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -394,39 +394,39 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -460,13 +460,13 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -823,11 +823,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -837,11 +837,11 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -851,11 +851,11 @@
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -865,94 +865,94 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
     </row>
     <row r="5" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
     </row>
     <row r="6" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18" t="s">
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="18" t="s">
+      <c r="J6" s="20" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="19" t="s">
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19" t="s">
+      <c r="D7" s="27"/>
+      <c r="E7" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19" t="s">
+      <c r="F7" s="27"/>
+      <c r="G7" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="19"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
     </row>
     <row r="8" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="20">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="28">
         <v>37500</v>
       </c>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20">
+      <c r="D8" s="28"/>
+      <c r="E8" s="28">
         <v>19500</v>
       </c>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20">
+      <c r="F8" s="28"/>
+      <c r="G8" s="28">
         <v>15000</v>
       </c>
-      <c r="H8" s="20"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
     </row>
     <row r="9" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="3" t="s">
         <v>13</v>
       </c>
@@ -971,8 +971,8 @@
       <c r="H9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
     </row>
     <row r="10" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
@@ -1339,10 +1339,10 @@
       <c r="J22" s="5"/>
     </row>
     <row r="23" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="18"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="3">
         <f t="shared" ref="C23:H23" si="4">SUM(C10:C22)</f>
         <v>0</v>
@@ -1374,43 +1374,49 @@
       <c r="J23" s="5"/>
     </row>
     <row r="25" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="24" t="s">
+      <c r="A25" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="24"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="25"/>
-      <c r="J25" s="25"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="22"/>
     </row>
     <row r="26" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H26" s="26" t="s">
+      <c r="H26" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="I26" s="26"/>
-      <c r="J26" s="26"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="23"/>
     </row>
     <row r="27" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D27" s="27" t="s">
+      <c r="D27" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="H27" s="27" t="s">
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="H27" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="I27" s="27"/>
+      <c r="I27" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="G8:H8"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A3:C3"/>
@@ -1427,12 +1433,6 @@
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="I6:I9"/>
     <mergeCell ref="J6:J9"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="G8:H8"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -1451,67 +1451,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="str">
+      <c r="A1" s="18" t="str">
         <f>'Sheet 1'!A1</f>
         <v>BỆNH VIỆN THAN - KHOÁNG SẢN</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
       <c r="D1" s="12"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="str">
+      <c r="A2" s="18" t="str">
         <f>'Sheet 1'!A2</f>
         <v>CƠ SỞ 2</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
       <c r="D2" s="12"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="18" t="str">
         <f>'Sheet 1'!A3</f>
         <v>KHOA YHCT-PHCN</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
       <c r="D3" s="12"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="21" t="str">
+      <c r="A4" s="24" t="str">
         <f>'Sheet 1'!A4</f>
         <v>BẢNG KÊ PHẪU THUẬT - THỦ THUẬT</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
       <c r="F4" s="15"/>
       <c r="G4" s="15"/>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="str">
+      <c r="A5" s="26" t="str">
         <f>'Sheet 1'!A5</f>
         <v>THÁNG….NĂM 2026</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B6" s="32" t="s">
@@ -1528,7 +1528,7 @@
       <c r="G6" s="13"/>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="19"/>
+      <c r="A7" s="27"/>
       <c r="B7" s="3" t="s">
         <v>30</v>
       </c>
@@ -1608,13 +1608,13 @@
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
     </row>
@@ -1630,17 +1630,17 @@
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="28" t="s">
+      <c r="D15" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="28"/>
+      <c r="E15" s="18"/>
       <c r="F15" s="12"/>
       <c r="G15" s="1"/>
     </row>
@@ -1677,12 +1677,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="str">
+      <c r="A1" s="18" t="str">
         <f>'Sheet 2'!A1</f>
         <v>BỆNH VIỆN THAN - KHOÁNG SẢN</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -1692,12 +1692,12 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="str">
+      <c r="A2" s="18" t="str">
         <f>'Sheet 2'!A2</f>
         <v>CƠ SỞ 2</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -1707,12 +1707,12 @@
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="18" t="str">
         <f>'Sheet 2'!A3</f>
         <v>KHOA YHCT-PHCN</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1722,34 +1722,34 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="21" t="str">
+      <c r="A4" s="24" t="str">
         <f>'Sheet 2'!A4</f>
         <v>BẢNG KÊ PHẪU THUẬT - THỦ THUẬT</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="str">
+      <c r="A5" s="40" t="str">
         <f>'Sheet 2'!A5</f>
         <v>THÁNG….NĂM 2026</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
+      <c r="B5" s="40"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -2093,54 +2093,86 @@
       <c r="A21" s="8"/>
     </row>
     <row r="22" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="24" t="s">
+      <c r="A22" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="24"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
     </row>
     <row r="23" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="8"/>
-      <c r="H23" s="40" t="s">
+      <c r="H23" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="I23" s="40"/>
-      <c r="J23" s="40"/>
+      <c r="I23" s="42"/>
+      <c r="J23" s="42"/>
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="27" t="s">
+      <c r="D24" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="H24" s="27" t="s">
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="H24" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="I24" s="27"/>
-      <c r="J24" s="27"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="68">
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="C22:J22"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:J13"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="G14:H14"/>
@@ -2157,48 +2189,16 @@
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="I9:J9"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>

</xml_diff>